<commit_message>
feat: import improved sub-schemas, more unit tests"
</commit_message>
<xml_diff>
--- a/project/excel/nist_ai_rmf.xlsx
+++ b/project/excel/nist_ai_rmf.xlsx
@@ -1446,17 +1446,17 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>trustworthiness_characteristic</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>addressed_by_actions</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>lifecycle_stage</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>trustworthiness_characteristic</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>addressed_by_actions</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
@@ -1500,10 +1500,10 @@
       <formula1>"IMMEDIATE,PROLONGED"</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"PLAN_AND_DESIGN,COLLECT_AND_PROCESS_DATA,BUILD_AND_USE_MODEL,VERIFY_AND_VALIDATE,DEPLOY_AND_USE,OPERATE_AND_MONITOR"</formula1>
-    </dataValidation>
-    <dataValidation sqref="G2:G1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"VALID_AND_RELIABLE,SAFE,SECURE_AND_RESILIENT,ACCOUNTABLE_AND_TRANSPARENT,EXPLAINABLE_AND_INTERPRETABLE,PRIVACY_ENHANCED,FAIR_WITH_HARMFUL_BIAS_MANAGED"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"DESIGN,DEVELOPMENT,DEPLOYMENT,OPERATION,DECOMMISSIONING"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1577,7 +1577,7 @@
       <formula1>"GV,MP,MS,MG"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"AI_DESIGN,AI_DEVELOPMENT,AI_DEPLOYMENT,OPERATION_AND_MONITORING,TEVV,HUMAN_FACTORS,DOMAIN_EXPERT,AI_IMPACT_ASSESSMENT,PROCUREMENT,GOVERNANCE_AND_OVERSIGHT,THIRD_PARTY_ENTITIES,END_USERS,AFFECTED_INDIVIDUALS_OR_COMMUNITIES,OTHER_AI_ACTORS,GENERAL_PUBLIC"</formula1>
+      <formula1>"GOVERNANCE_AND_OVERSIGHT,AI_DESIGN,AI_DEVELOPMENT,AI_DEPLOYMENT,AI_IMPACT_ASSESSMENT,OPERATION_AND_MONITORING,TEVV,DOMAIN_EXPERTS,END_USERS,HUMAN_FACTORS,AFFECTED_INDIVIDUALS_AND_COMMUNITIES,PROCUREMENT,THIRD_PARTY_ENTITIES"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1651,9 +1651,12 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"GOVERNANCE,PRE_DEPLOYMENT_TESTING,CONTENT_PROVENANCE,INCIDENT_DISCLOSURE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"DIGITAL_WATERMARKING,METADATA_RECORDING,DIGITAL_FINGERPRINTING,HUMAN_AUTHENTICATION"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1832,7 +1835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1858,61 +1861,31 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>profile_type</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>current_state</t>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>name</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>target_state</t>
+          <t>title</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>sector</t>
+          <t>description</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>addresses</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>see_also</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"USE_CASE,TEMPORAL_CURRENT,TEMPORAL_TARGET,CROSS_SECTORAL"</formula1>
-    </dataValidation>
-  </dataValidations>
+          <t>see_also</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2001,22 +1974,22 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>task_kind</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>typical_actors</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>lifecycle_stage</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ai_dimension</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>task_kind</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>typical_actors</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -2048,13 +2021,13 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"AI_DESIGN,AI_DEVELOPMENT,AI_DEPLOYMENT,OPERATION_AND_MONITORING,TEVV,HUMAN_FACTORS,DOMAIN_EXPERT,AI_IMPACT_ASSESSMENT,PROCUREMENT,GOVERNANCE_AND_OVERSIGHT,THIRD_PARTY_ENTITIES,END_USERS,AFFECTED_INDIVIDUALS_OR_COMMUNITIES,OTHER_AI_ACTORS,GENERAL_PUBLIC"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PLAN_AND_DESIGN,COLLECT_AND_PROCESS_DATA,BUILD_AND_USE_MODEL,VERIFY_AND_VALIDATE,DEPLOY_AND_USE,OPERATE_AND_MONITOR"</formula1>
     </dataValidation>
-    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"APPLICATION_CONTEXT,DATA_AND_INPUT,AI_MODEL,TASK_AND_OUTPUT,PEOPLE_AND_PLANET"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"AI_DESIGN,AI_DEVELOPMENT,AI_DEPLOYMENT,OPERATION_AND_MONITORING,TEVV,HUMAN_FACTORS,DOMAIN_EXPERT,AI_IMPACT_ASSESSMENT,PROCUREMENT,GOVERNANCE_AND_OVERSIGHT,THIRD_PARTY_ENTITIES,END_USERS,AFFECTED_INDIVIDUALS_OR_COMMUNITIES,OTHER_AI_ACTORS,GENERAL_PUBLIC"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>